<commit_message>
Fix banda gpon fixa
</commit_message>
<xml_diff>
--- a/arquivos/capacity_fixa.xlsx
+++ b/arquivos/capacity_fixa.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\F257064\Documents\Codes\NEW_NFV\arquivos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\F257064\Documents\Codes\atualizacao nfv automatico\NEW_NFV\arquivos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{632D1099-31E8-4928-AAAC-C6D13585EC27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5097C5B-269D-4194-A461-57B1FD371219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24" yWindow="24" windowWidth="22992" windowHeight="12216" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-24120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
@@ -3264,7 +3264,7 @@
         <v>10</v>
       </c>
       <c r="F3" s="1">
-        <v>890.53241910000008</v>
+        <v>200</v>
       </c>
       <c r="G3" t="s">
         <v>687</v>
@@ -3333,7 +3333,7 @@
         <v>10</v>
       </c>
       <c r="F6" s="1">
-        <v>928.91892144999997</v>
+        <v>200</v>
       </c>
       <c r="G6" t="s">
         <v>529</v>
@@ -3379,7 +3379,7 @@
         <v>10</v>
       </c>
       <c r="F8" s="1">
-        <v>959.57883548999996</v>
+        <v>200</v>
       </c>
       <c r="G8" t="s">
         <v>529</v>
@@ -3402,7 +3402,7 @@
         <v>10</v>
       </c>
       <c r="F9" s="1">
-        <v>981.00946372999999</v>
+        <v>200</v>
       </c>
       <c r="G9" t="s">
         <v>529</v>
@@ -3448,7 +3448,7 @@
         <v>10</v>
       </c>
       <c r="F11" s="1">
-        <v>882.17617970000003</v>
+        <v>200</v>
       </c>
       <c r="G11" t="s">
         <v>529</v>
@@ -3540,7 +3540,7 @@
         <v>10</v>
       </c>
       <c r="F15" s="1">
-        <v>701.23374890000002</v>
+        <v>200</v>
       </c>
       <c r="G15" t="s">
         <v>362</v>
@@ -3586,7 +3586,7 @@
         <v>10</v>
       </c>
       <c r="F17" s="1">
-        <v>757.07636079999997</v>
+        <v>200</v>
       </c>
       <c r="G17" t="s">
         <v>362</v>
@@ -3655,7 +3655,7 @@
         <v>10</v>
       </c>
       <c r="F20" s="1">
-        <v>889.01230090000001</v>
+        <v>200</v>
       </c>
       <c r="G20" t="s">
         <v>321</v>
@@ -3747,7 +3747,7 @@
         <v>10</v>
       </c>
       <c r="F24" s="1">
-        <v>1813.9276125700001</v>
+        <v>200</v>
       </c>
       <c r="G24" t="s">
         <v>529</v>
@@ -3770,7 +3770,7 @@
         <v>10</v>
       </c>
       <c r="F25" s="1">
-        <v>718.04160130000002</v>
+        <v>200</v>
       </c>
       <c r="G25" t="s">
         <v>388</v>
@@ -3839,7 +3839,7 @@
         <v>10</v>
       </c>
       <c r="F28" s="1">
-        <v>905.27678400000002</v>
+        <v>200</v>
       </c>
       <c r="G28" t="s">
         <v>899</v>
@@ -4092,7 +4092,7 @@
         <v>10</v>
       </c>
       <c r="F39" s="1">
-        <v>511.95407610000001</v>
+        <v>200</v>
       </c>
       <c r="G39" t="s">
         <v>351</v>
@@ -4138,7 +4138,7 @@
         <v>10</v>
       </c>
       <c r="F41" s="1">
-        <v>707.09351479999998</v>
+        <v>200</v>
       </c>
       <c r="G41" t="s">
         <v>351</v>
@@ -4161,7 +4161,7 @@
         <v>10</v>
       </c>
       <c r="F42" s="1">
-        <v>964.05682973</v>
+        <v>200</v>
       </c>
       <c r="G42" t="s">
         <v>578</v>
@@ -4230,7 +4230,7 @@
         <v>10</v>
       </c>
       <c r="F45" s="1">
-        <v>937.74067184</v>
+        <v>200</v>
       </c>
       <c r="G45" t="s">
         <v>388</v>
@@ -4253,7 +4253,7 @@
         <v>10</v>
       </c>
       <c r="F46" s="1">
-        <v>640.98953729999994</v>
+        <v>200</v>
       </c>
       <c r="G46" t="s">
         <v>651</v>
@@ -4299,7 +4299,7 @@
         <v>10</v>
       </c>
       <c r="F48" s="1">
-        <v>981.18008395999993</v>
+        <v>200</v>
       </c>
       <c r="G48" t="s">
         <v>351</v>
@@ -4368,7 +4368,7 @@
         <v>10</v>
       </c>
       <c r="F51" s="1">
-        <v>805.41846959999998</v>
+        <v>200</v>
       </c>
       <c r="G51" t="s">
         <v>351</v>
@@ -4414,7 +4414,7 @@
         <v>10</v>
       </c>
       <c r="F53" s="1">
-        <v>683.32461210000008</v>
+        <v>200</v>
       </c>
       <c r="G53" t="s">
         <v>351</v>
@@ -4437,7 +4437,7 @@
         <v>10</v>
       </c>
       <c r="F54" s="1">
-        <v>735.38224539999999</v>
+        <v>200</v>
       </c>
       <c r="G54" t="s">
         <v>351</v>
@@ -4460,7 +4460,7 @@
         <v>10</v>
       </c>
       <c r="F55" s="1">
-        <v>1806.3462424436239</v>
+        <v>200</v>
       </c>
       <c r="G55" t="s">
         <v>351</v>
@@ -4483,7 +4483,7 @@
         <v>10</v>
       </c>
       <c r="F56" s="1">
-        <v>842.00992659999997</v>
+        <v>200</v>
       </c>
       <c r="G56" t="s">
         <v>351</v>
@@ -4506,7 +4506,7 @@
         <v>10</v>
       </c>
       <c r="F57" s="1">
-        <v>1588.1948490900002</v>
+        <v>200</v>
       </c>
       <c r="G57" t="s">
         <v>351</v>
@@ -4552,7 +4552,7 @@
         <v>10</v>
       </c>
       <c r="F59" s="1">
-        <v>1890.3112630515002</v>
+        <v>200</v>
       </c>
       <c r="G59" t="s">
         <v>351</v>
@@ -4621,7 +4621,7 @@
         <v>10</v>
       </c>
       <c r="F62" s="1">
-        <v>647.90110600000003</v>
+        <v>200</v>
       </c>
       <c r="G62" t="s">
         <v>351</v>
@@ -4667,7 +4667,7 @@
         <v>10</v>
       </c>
       <c r="F64" s="1">
-        <v>648.86410810000007</v>
+        <v>200</v>
       </c>
       <c r="G64" t="s">
         <v>351</v>
@@ -4713,7 +4713,7 @@
         <v>10</v>
       </c>
       <c r="F66" s="1">
-        <v>1642.11314159208</v>
+        <v>200</v>
       </c>
       <c r="G66" t="s">
         <v>351</v>
@@ -4759,7 +4759,7 @@
         <v>10</v>
       </c>
       <c r="F68" s="1">
-        <v>862.88580609999997</v>
+        <v>200</v>
       </c>
       <c r="G68" t="s">
         <v>351</v>
@@ -4828,7 +4828,7 @@
         <v>10</v>
       </c>
       <c r="F71" s="1">
-        <v>849.97093599999994</v>
+        <v>200</v>
       </c>
       <c r="G71" t="s">
         <v>362</v>
@@ -4874,7 +4874,7 @@
         <v>10</v>
       </c>
       <c r="F73" s="1">
-        <v>925.43812736999996</v>
+        <v>200</v>
       </c>
       <c r="G73" t="s">
         <v>362</v>
@@ -4920,7 +4920,7 @@
         <v>10</v>
       </c>
       <c r="F75" s="1">
-        <v>885.55719790000001</v>
+        <v>200</v>
       </c>
       <c r="G75" t="s">
         <v>362</v>
@@ -5012,7 +5012,7 @@
         <v>10</v>
       </c>
       <c r="F79" s="1">
-        <v>809.82332330000008</v>
+        <v>200</v>
       </c>
       <c r="G79" t="s">
         <v>362</v>
@@ -5035,7 +5035,7 @@
         <v>10</v>
       </c>
       <c r="F80" s="1">
-        <v>793.02609340000004</v>
+        <v>200</v>
       </c>
       <c r="G80" t="s">
         <v>362</v>
@@ -5081,7 +5081,7 @@
         <v>10</v>
       </c>
       <c r="F82" s="1">
-        <v>793.16059220000011</v>
+        <v>200</v>
       </c>
       <c r="G82" t="s">
         <v>362</v>
@@ -5127,7 +5127,7 @@
         <v>10</v>
       </c>
       <c r="F84" s="1">
-        <v>830.48630239999989</v>
+        <v>200</v>
       </c>
       <c r="G84" t="s">
         <v>362</v>
@@ -5173,7 +5173,7 @@
         <v>10</v>
       </c>
       <c r="F86" s="1">
-        <v>643.8234367</v>
+        <v>200</v>
       </c>
       <c r="G86" t="s">
         <v>362</v>
@@ -5242,7 +5242,7 @@
         <v>10</v>
       </c>
       <c r="F89" s="1">
-        <v>835.16791599999999</v>
+        <v>200</v>
       </c>
       <c r="G89" t="s">
         <v>519</v>
@@ -5334,7 +5334,7 @@
         <v>10</v>
       </c>
       <c r="F93" s="1">
-        <v>846.07879630000002</v>
+        <v>200</v>
       </c>
       <c r="G93" t="s">
         <v>519</v>
@@ -5380,7 +5380,7 @@
         <v>10</v>
       </c>
       <c r="F95" s="1">
-        <v>2400.2009215700004</v>
+        <v>200</v>
       </c>
       <c r="G95" t="s">
         <v>373</v>
@@ -5495,7 +5495,7 @@
         <v>10</v>
       </c>
       <c r="F100" s="1">
-        <v>1696.1928437899999</v>
+        <v>200</v>
       </c>
       <c r="G100" t="s">
         <v>373</v>
@@ -5771,7 +5771,7 @@
         <v>10</v>
       </c>
       <c r="F112" s="1">
-        <v>1414.80723964649</v>
+        <v>200</v>
       </c>
       <c r="G112" t="s">
         <v>388</v>
@@ -5932,7 +5932,7 @@
         <v>10</v>
       </c>
       <c r="F119" s="1">
-        <v>643.20916050000005</v>
+        <v>200</v>
       </c>
       <c r="G119" t="s">
         <v>395</v>
@@ -5978,7 +5978,7 @@
         <v>10</v>
       </c>
       <c r="F121" s="1">
-        <v>924.35522150000008</v>
+        <v>200</v>
       </c>
       <c r="G121" t="s">
         <v>395</v>
@@ -6024,7 +6024,7 @@
         <v>10</v>
       </c>
       <c r="F123" s="1">
-        <v>236.76519269999997</v>
+        <v>200</v>
       </c>
       <c r="G123" t="s">
         <v>395</v>
@@ -6070,7 +6070,7 @@
         <v>10</v>
       </c>
       <c r="F125" s="1">
-        <v>816.34630799999991</v>
+        <v>200</v>
       </c>
       <c r="G125" t="s">
         <v>395</v>
@@ -6093,7 +6093,7 @@
         <v>10</v>
       </c>
       <c r="F126" s="1">
-        <v>932.43298916999993</v>
+        <v>200</v>
       </c>
       <c r="G126" t="s">
         <v>388</v>
@@ -6254,7 +6254,7 @@
         <v>10</v>
       </c>
       <c r="F133" s="1">
-        <v>828.03541710000002</v>
+        <v>200</v>
       </c>
       <c r="G133" t="s">
         <v>855</v>
@@ -6507,7 +6507,7 @@
         <v>10</v>
       </c>
       <c r="F144" s="1">
-        <v>900.36789292000003</v>
+        <v>200</v>
       </c>
       <c r="G144" t="s">
         <v>408</v>
@@ -6645,7 +6645,7 @@
         <v>10</v>
       </c>
       <c r="F150" s="1">
-        <v>473.57539939999998</v>
+        <v>200</v>
       </c>
       <c r="G150" t="s">
         <v>420</v>
@@ -6691,7 +6691,7 @@
         <v>10</v>
       </c>
       <c r="F152" s="1">
-        <v>503.26186090000004</v>
+        <v>200</v>
       </c>
       <c r="G152" t="s">
         <v>420</v>
@@ -6806,7 +6806,7 @@
         <v>10</v>
       </c>
       <c r="F157" s="1">
-        <v>947.27181376999999</v>
+        <v>200</v>
       </c>
       <c r="G157" t="s">
         <v>918</v>
@@ -6852,7 +6852,7 @@
         <v>10</v>
       </c>
       <c r="F159" s="1">
-        <v>9935.1704618100011</v>
+        <v>200</v>
       </c>
       <c r="G159" t="s">
         <v>519</v>
@@ -6921,7 +6921,7 @@
         <v>10</v>
       </c>
       <c r="F162" s="1">
-        <v>793.93926910000005</v>
+        <v>200</v>
       </c>
       <c r="G162" t="s">
         <v>429</v>
@@ -6944,7 +6944,7 @@
         <v>10</v>
       </c>
       <c r="F163" s="1">
-        <v>540.24292479999997</v>
+        <v>200</v>
       </c>
       <c r="G163" t="s">
         <v>429</v>
@@ -6990,7 +6990,7 @@
         <v>10</v>
       </c>
       <c r="F165" s="1">
-        <v>678.89151779999997</v>
+        <v>200</v>
       </c>
       <c r="G165" t="s">
         <v>429</v>
@@ -7036,7 +7036,7 @@
         <v>10</v>
       </c>
       <c r="F167" s="1">
-        <v>781.44867969999996</v>
+        <v>200</v>
       </c>
       <c r="G167" t="s">
         <v>429</v>
@@ -7059,7 +7059,7 @@
         <v>10</v>
       </c>
       <c r="F168" s="1">
-        <v>893.07540599999993</v>
+        <v>200</v>
       </c>
       <c r="G168" t="s">
         <v>855</v>
@@ -7082,7 +7082,7 @@
         <v>10</v>
       </c>
       <c r="F169" s="1">
-        <v>969.10254729999997</v>
+        <v>200</v>
       </c>
       <c r="G169" t="s">
         <v>687</v>
@@ -7128,7 +7128,7 @@
         <v>10</v>
       </c>
       <c r="F171" s="1">
-        <v>824.4680955</v>
+        <v>200</v>
       </c>
       <c r="G171" t="s">
         <v>578</v>
@@ -7220,7 +7220,7 @@
         <v>10</v>
       </c>
       <c r="F175" s="1">
-        <v>528.15879770000004</v>
+        <v>200</v>
       </c>
       <c r="G175" t="s">
         <v>644</v>
@@ -7335,7 +7335,7 @@
         <v>10</v>
       </c>
       <c r="F180" s="1">
-        <v>962.78838807999989</v>
+        <v>200</v>
       </c>
       <c r="G180" t="s">
         <v>918</v>
@@ -7404,7 +7404,7 @@
         <v>10</v>
       </c>
       <c r="F183" s="1">
-        <v>266.7514865</v>
+        <v>200</v>
       </c>
       <c r="G183" t="s">
         <v>443</v>
@@ -7450,7 +7450,7 @@
         <v>10</v>
       </c>
       <c r="F185" s="1">
-        <v>866.3877483</v>
+        <v>200</v>
       </c>
       <c r="G185" t="s">
         <v>443</v>
@@ -7473,7 +7473,7 @@
         <v>10</v>
       </c>
       <c r="F186" s="1">
-        <v>924.48128596999993</v>
+        <v>200</v>
       </c>
       <c r="G186" t="s">
         <v>443</v>
@@ -7542,7 +7542,7 @@
         <v>10</v>
       </c>
       <c r="F189" s="1">
-        <v>887.60493719999999</v>
+        <v>200</v>
       </c>
       <c r="G189" t="s">
         <v>713</v>
@@ -7726,7 +7726,7 @@
         <v>10</v>
       </c>
       <c r="F197" s="1">
-        <v>713.27301629999999</v>
+        <v>200</v>
       </c>
       <c r="G197" t="s">
         <v>469</v>
@@ -7772,7 +7772,7 @@
         <v>10</v>
       </c>
       <c r="F199" s="1">
-        <v>673.9653148000001</v>
+        <v>200</v>
       </c>
       <c r="G199" t="s">
         <v>465</v>
@@ -7818,7 +7818,7 @@
         <v>10</v>
       </c>
       <c r="F201" s="1">
-        <v>945.14318175999995</v>
+        <v>200</v>
       </c>
       <c r="G201" t="s">
         <v>465</v>
@@ -7910,7 +7910,7 @@
         <v>10</v>
       </c>
       <c r="F205" s="1">
-        <v>831.97061970000004</v>
+        <v>200</v>
       </c>
       <c r="G205" t="s">
         <v>469</v>
@@ -7956,7 +7956,7 @@
         <v>10</v>
       </c>
       <c r="F207" s="1">
-        <v>721.9183835</v>
+        <v>200</v>
       </c>
       <c r="G207" t="s">
         <v>469</v>
@@ -8002,7 +8002,7 @@
         <v>10</v>
       </c>
       <c r="F209" s="1">
-        <v>402.1183661</v>
+        <v>200</v>
       </c>
       <c r="G209" t="s">
         <v>463</v>
@@ -8048,7 +8048,7 @@
         <v>10</v>
       </c>
       <c r="F211" s="1">
-        <v>867.55802989999995</v>
+        <v>200</v>
       </c>
       <c r="G211" t="s">
         <v>469</v>
@@ -8140,7 +8140,7 @@
         <v>10</v>
       </c>
       <c r="F215" s="1">
-        <v>917.60063708999996</v>
+        <v>200</v>
       </c>
       <c r="G215" t="s">
         <v>469</v>
@@ -8232,7 +8232,7 @@
         <v>10</v>
       </c>
       <c r="F219" s="1">
-        <v>925.24660131000007</v>
+        <v>200</v>
       </c>
       <c r="G219" t="s">
         <v>469</v>
@@ -8278,7 +8278,7 @@
         <v>10</v>
       </c>
       <c r="F221" s="1">
-        <v>888.11464030000002</v>
+        <v>200</v>
       </c>
       <c r="G221" t="s">
         <v>753</v>
@@ -8324,7 +8324,7 @@
         <v>10</v>
       </c>
       <c r="F223" s="1">
-        <v>696.24690740000005</v>
+        <v>200</v>
       </c>
       <c r="G223" t="s">
         <v>519</v>
@@ -8370,7 +8370,7 @@
         <v>10</v>
       </c>
       <c r="F225" s="1">
-        <v>976.22041836000005</v>
+        <v>200</v>
       </c>
       <c r="G225" t="s">
         <v>503</v>
@@ -8554,7 +8554,7 @@
         <v>10</v>
       </c>
       <c r="F233" s="1">
-        <v>752.5596084</v>
+        <v>200</v>
       </c>
       <c r="G233" t="s">
         <v>351</v>
@@ -8623,7 +8623,7 @@
         <v>10</v>
       </c>
       <c r="F236" s="1">
-        <v>979.42577275999997</v>
+        <v>200</v>
       </c>
       <c r="G236" t="s">
         <v>503</v>
@@ -8715,7 +8715,7 @@
         <v>10</v>
       </c>
       <c r="F240" s="1">
-        <v>989.41410088000009</v>
+        <v>200</v>
       </c>
       <c r="G240" t="s">
         <v>855</v>
@@ -8738,7 +8738,7 @@
         <v>10</v>
       </c>
       <c r="F241" s="1">
-        <v>895.44711319999999</v>
+        <v>200</v>
       </c>
       <c r="G241" t="s">
         <v>855</v>
@@ -8761,7 +8761,7 @@
         <v>10</v>
       </c>
       <c r="F242" s="1">
-        <v>979.41086199000006</v>
+        <v>200</v>
       </c>
       <c r="G242" t="s">
         <v>503</v>
@@ -8807,7 +8807,7 @@
         <v>10</v>
       </c>
       <c r="F244" s="1">
-        <v>901.97171187000004</v>
+        <v>200</v>
       </c>
       <c r="G244" t="s">
         <v>503</v>
@@ -8853,7 +8853,7 @@
         <v>10</v>
       </c>
       <c r="F246" s="1">
-        <v>835.67136440000002</v>
+        <v>200</v>
       </c>
       <c r="G246" t="s">
         <v>503</v>
@@ -8899,7 +8899,7 @@
         <v>10</v>
       </c>
       <c r="F248" s="1">
-        <v>947.41741612999999</v>
+        <v>200</v>
       </c>
       <c r="G248" t="s">
         <v>503</v>
@@ -8945,7 +8945,7 @@
         <v>10</v>
       </c>
       <c r="F250" s="1">
-        <v>949.66428517000008</v>
+        <v>200</v>
       </c>
       <c r="G250" t="s">
         <v>503</v>
@@ -8991,7 +8991,7 @@
         <v>10</v>
       </c>
       <c r="F252" s="1">
-        <v>863.02296699999999</v>
+        <v>200</v>
       </c>
       <c r="G252" t="s">
         <v>503</v>
@@ -9037,7 +9037,7 @@
         <v>10</v>
       </c>
       <c r="F254" s="1">
-        <v>802.01825450000001</v>
+        <v>200</v>
       </c>
       <c r="G254" t="s">
         <v>503</v>
@@ -9083,7 +9083,7 @@
         <v>10</v>
       </c>
       <c r="F256" s="1">
-        <v>823.24606970000002</v>
+        <v>200</v>
       </c>
       <c r="G256" t="s">
         <v>503</v>
@@ -9129,7 +9129,7 @@
         <v>10</v>
       </c>
       <c r="F258" s="1">
-        <v>890.23141319999991</v>
+        <v>200</v>
       </c>
       <c r="G258" t="s">
         <v>503</v>
@@ -9175,7 +9175,7 @@
         <v>10</v>
       </c>
       <c r="F260" s="1">
-        <v>905.04618431999995</v>
+        <v>200</v>
       </c>
       <c r="G260" t="s">
         <v>503</v>
@@ -9221,7 +9221,7 @@
         <v>10</v>
       </c>
       <c r="F262" s="1">
-        <v>905.31245452999997</v>
+        <v>200</v>
       </c>
       <c r="G262" t="s">
         <v>503</v>
@@ -9290,7 +9290,7 @@
         <v>10</v>
       </c>
       <c r="F265" s="1">
-        <v>940.02608722000002</v>
+        <v>200</v>
       </c>
       <c r="G265" t="s">
         <v>503</v>
@@ -9336,7 +9336,7 @@
         <v>10</v>
       </c>
       <c r="F267" s="1">
-        <v>971.73206391999997</v>
+        <v>200</v>
       </c>
       <c r="G267" t="s">
         <v>503</v>
@@ -9405,7 +9405,7 @@
         <v>10</v>
       </c>
       <c r="F270" s="1">
-        <v>949.86933368999996</v>
+        <v>200</v>
       </c>
       <c r="G270" t="s">
         <v>503</v>
@@ -9451,7 +9451,7 @@
         <v>10</v>
       </c>
       <c r="F272" s="1">
-        <v>913.10857352999994</v>
+        <v>200</v>
       </c>
       <c r="G272" t="s">
         <v>503</v>
@@ -9497,7 +9497,7 @@
         <v>10</v>
       </c>
       <c r="F274" s="1">
-        <v>963.60930284000005</v>
+        <v>200</v>
       </c>
       <c r="G274" t="s">
         <v>503</v>
@@ -9543,7 +9543,7 @@
         <v>10</v>
       </c>
       <c r="F276" s="1">
-        <v>998.20242280399998</v>
+        <v>200</v>
       </c>
       <c r="G276" t="s">
         <v>503</v>
@@ -9612,7 +9612,7 @@
         <v>10</v>
       </c>
       <c r="F279" s="1">
-        <v>995.93169434100002</v>
+        <v>200</v>
       </c>
       <c r="G279" t="s">
         <v>503</v>
@@ -9911,7 +9911,7 @@
         <v>10</v>
       </c>
       <c r="F292" s="1">
-        <v>766.19308960000012</v>
+        <v>200</v>
       </c>
       <c r="G292" t="s">
         <v>519</v>
@@ -10003,7 +10003,7 @@
         <v>10</v>
       </c>
       <c r="F296" s="1">
-        <v>1011.8142636700001</v>
+        <v>200</v>
       </c>
       <c r="G296" t="s">
         <v>651</v>
@@ -10049,7 +10049,7 @@
         <v>10</v>
       </c>
       <c r="F298" s="1">
-        <v>1581.5568291</v>
+        <v>200</v>
       </c>
       <c r="G298" t="s">
         <v>777</v>
@@ -10118,7 +10118,7 @@
         <v>10</v>
       </c>
       <c r="F301" s="1">
-        <v>614.70494840000003</v>
+        <v>200</v>
       </c>
       <c r="G301" t="s">
         <v>529</v>
@@ -10187,7 +10187,7 @@
         <v>10</v>
       </c>
       <c r="F304" s="1">
-        <v>718.10732939999991</v>
+        <v>200</v>
       </c>
       <c r="G304" t="s">
         <v>529</v>
@@ -10233,7 +10233,7 @@
         <v>10</v>
       </c>
       <c r="F306" s="1">
-        <v>627.0695048</v>
+        <v>200</v>
       </c>
       <c r="G306" t="s">
         <v>529</v>
@@ -10279,7 +10279,7 @@
         <v>10</v>
       </c>
       <c r="F308" s="1">
-        <v>531.28208480000012</v>
+        <v>200</v>
       </c>
       <c r="G308" t="s">
         <v>529</v>
@@ -10302,7 +10302,7 @@
         <v>10</v>
       </c>
       <c r="F309" s="1">
-        <v>602.90245549999997</v>
+        <v>200</v>
       </c>
       <c r="G309" t="s">
         <v>529</v>
@@ -10394,7 +10394,7 @@
         <v>10</v>
       </c>
       <c r="F313" s="1">
-        <v>955.70064599</v>
+        <v>200</v>
       </c>
       <c r="G313" t="s">
         <v>918</v>
@@ -10463,7 +10463,7 @@
         <v>10</v>
       </c>
       <c r="F316" s="1">
-        <v>644.99032389999991</v>
+        <v>200</v>
       </c>
       <c r="G316" t="s">
         <v>855</v>
@@ -10509,7 +10509,7 @@
         <v>10</v>
       </c>
       <c r="F318" s="1">
-        <v>728.11474929999997</v>
+        <v>200</v>
       </c>
       <c r="G318" t="s">
         <v>855</v>
@@ -10624,7 +10624,7 @@
         <v>10</v>
       </c>
       <c r="F323" s="1">
-        <v>927.86428344000001</v>
+        <v>200</v>
       </c>
       <c r="G323" t="s">
         <v>669</v>
@@ -10693,7 +10693,7 @@
         <v>10</v>
       </c>
       <c r="F326" s="1">
-        <v>803.83502420000002</v>
+        <v>200</v>
       </c>
       <c r="G326" t="s">
         <v>543</v>
@@ -10808,7 +10808,7 @@
         <v>10</v>
       </c>
       <c r="F331" s="1">
-        <v>780.04888329999994</v>
+        <v>200</v>
       </c>
       <c r="G331" t="s">
         <v>519</v>
@@ -10854,7 +10854,7 @@
         <v>10</v>
       </c>
       <c r="F333" s="1">
-        <v>889.11944099999994</v>
+        <v>200</v>
       </c>
       <c r="G333" t="s">
         <v>855</v>
@@ -10923,7 +10923,7 @@
         <v>10</v>
       </c>
       <c r="F336" s="1">
-        <v>640.56188859999997</v>
+        <v>200</v>
       </c>
       <c r="G336" t="s">
         <v>408</v>
@@ -11038,7 +11038,7 @@
         <v>10</v>
       </c>
       <c r="F341" s="1">
-        <v>972.69845303</v>
+        <v>200</v>
       </c>
       <c r="G341" t="s">
         <v>429</v>
@@ -11084,7 +11084,7 @@
         <v>10</v>
       </c>
       <c r="F343" s="1">
-        <v>859.42411829999992</v>
+        <v>200</v>
       </c>
       <c r="G343" t="s">
         <v>651</v>
@@ -11176,7 +11176,7 @@
         <v>10</v>
       </c>
       <c r="F347" s="1">
-        <v>883.85657300000003</v>
+        <v>200</v>
       </c>
       <c r="G347" t="s">
         <v>687</v>
@@ -11222,7 +11222,7 @@
         <v>10</v>
       </c>
       <c r="F349" s="1">
-        <v>922.16030405000004</v>
+        <v>200</v>
       </c>
       <c r="G349" t="s">
         <v>687</v>
@@ -11452,7 +11452,7 @@
         <v>10</v>
       </c>
       <c r="F359" s="1">
-        <v>825.14290800000003</v>
+        <v>200</v>
       </c>
       <c r="G359" t="s">
         <v>687</v>
@@ -11498,7 +11498,7 @@
         <v>10</v>
       </c>
       <c r="F361" s="1">
-        <v>502.93060050000003</v>
+        <v>200</v>
       </c>
       <c r="G361" t="s">
         <v>567</v>
@@ -11544,7 +11544,7 @@
         <v>10</v>
       </c>
       <c r="F363" s="1">
-        <v>852.99485709999999</v>
+        <v>200</v>
       </c>
       <c r="G363" t="s">
         <v>567</v>
@@ -11567,7 +11567,7 @@
         <v>10</v>
       </c>
       <c r="F364" s="1">
-        <v>858.46999380000011</v>
+        <v>200</v>
       </c>
       <c r="G364" t="s">
         <v>519</v>
@@ -11682,7 +11682,7 @@
         <v>10</v>
       </c>
       <c r="F369" s="1">
-        <v>895.25475610000001</v>
+        <v>200</v>
       </c>
       <c r="G369" t="s">
         <v>578</v>
@@ -11705,7 +11705,7 @@
         <v>10</v>
       </c>
       <c r="F370" s="1">
-        <v>902.00553110999999</v>
+        <v>200</v>
       </c>
       <c r="G370" t="s">
         <v>578</v>
@@ -11728,7 +11728,7 @@
         <v>10</v>
       </c>
       <c r="F371" s="1">
-        <v>891.72924159999991</v>
+        <v>200</v>
       </c>
       <c r="G371" t="s">
         <v>578</v>
@@ -11751,7 +11751,7 @@
         <v>10</v>
       </c>
       <c r="F372" s="1">
-        <v>870.9874208</v>
+        <v>200</v>
       </c>
       <c r="G372" t="s">
         <v>578</v>
@@ -11774,7 +11774,7 @@
         <v>10</v>
       </c>
       <c r="F373" s="1">
-        <v>843.06105160000004</v>
+        <v>200</v>
       </c>
       <c r="G373" t="s">
         <v>578</v>
@@ -11889,7 +11889,7 @@
         <v>10</v>
       </c>
       <c r="F378" s="1">
-        <v>711.61307890000012</v>
+        <v>200</v>
       </c>
       <c r="G378" t="s">
         <v>519</v>
@@ -11935,7 +11935,7 @@
         <v>10</v>
       </c>
       <c r="F380" s="1">
-        <v>982.37117235999995</v>
+        <v>200</v>
       </c>
       <c r="G380" t="s">
         <v>519</v>
@@ -11958,7 +11958,7 @@
         <v>10</v>
       </c>
       <c r="F381" s="1">
-        <v>304.82323419999989</v>
+        <v>200</v>
       </c>
       <c r="G381" t="s">
         <v>584</v>
@@ -12027,7 +12027,7 @@
         <v>10</v>
       </c>
       <c r="F384" s="1">
-        <v>741.27526139999998</v>
+        <v>200</v>
       </c>
       <c r="G384" t="s">
         <v>388</v>
@@ -12050,7 +12050,7 @@
         <v>10</v>
       </c>
       <c r="F385" s="1">
-        <v>827.05555549999997</v>
+        <v>200</v>
       </c>
       <c r="G385" t="s">
         <v>777</v>
@@ -12165,7 +12165,7 @@
         <v>10</v>
       </c>
       <c r="F390" s="1">
-        <v>890.470191</v>
+        <v>200</v>
       </c>
       <c r="G390" t="s">
         <v>388</v>
@@ -12188,7 +12188,7 @@
         <v>10</v>
       </c>
       <c r="F391" s="1">
-        <v>865.0610107</v>
+        <v>200</v>
       </c>
       <c r="G391" t="s">
         <v>651</v>
@@ -12257,7 +12257,7 @@
         <v>10</v>
       </c>
       <c r="F394" s="1">
-        <v>917.23833479999996</v>
+        <v>200</v>
       </c>
       <c r="G394" t="s">
         <v>918</v>
@@ -12280,7 +12280,7 @@
         <v>10</v>
       </c>
       <c r="F395" s="1">
-        <v>863.41480139999999</v>
+        <v>200</v>
       </c>
       <c r="G395" t="s">
         <v>408</v>
@@ -12326,7 +12326,7 @@
         <v>10</v>
       </c>
       <c r="F397" s="1">
-        <v>912.38771411000005</v>
+        <v>200</v>
       </c>
       <c r="G397" t="s">
         <v>420</v>
@@ -12395,7 +12395,7 @@
         <v>10</v>
       </c>
       <c r="F400" s="1">
-        <v>803.95178190000001</v>
+        <v>200</v>
       </c>
       <c r="G400" t="s">
         <v>713</v>
@@ -12441,7 +12441,7 @@
         <v>10</v>
       </c>
       <c r="F402" s="1">
-        <v>785.94808799999998</v>
+        <v>200</v>
       </c>
       <c r="G402" t="s">
         <v>713</v>
@@ -12487,7 +12487,7 @@
         <v>10</v>
       </c>
       <c r="F404" s="1">
-        <v>539.27080820000003</v>
+        <v>200</v>
       </c>
       <c r="G404" t="s">
         <v>351</v>
@@ -12510,7 +12510,7 @@
         <v>10</v>
       </c>
       <c r="F405" s="1">
-        <v>882.55842469999993</v>
+        <v>200</v>
       </c>
       <c r="G405" t="s">
         <v>606</v>
@@ -12533,7 +12533,7 @@
         <v>10</v>
       </c>
       <c r="F406" s="1">
-        <v>891.80050199999994</v>
+        <v>200</v>
       </c>
       <c r="G406" t="s">
         <v>606</v>
@@ -12556,7 +12556,7 @@
         <v>10</v>
       </c>
       <c r="F407" s="1">
-        <v>738.66283989999999</v>
+        <v>200</v>
       </c>
       <c r="G407" t="s">
         <v>606</v>
@@ -12602,7 +12602,7 @@
         <v>10</v>
       </c>
       <c r="F409" s="1">
-        <v>817.82627799999989</v>
+        <v>200</v>
       </c>
       <c r="G409" t="s">
         <v>606</v>
@@ -12625,7 +12625,7 @@
         <v>10</v>
       </c>
       <c r="F410" s="1">
-        <v>954.72138670000004</v>
+        <v>200</v>
       </c>
       <c r="G410" t="s">
         <v>503</v>
@@ -12694,7 +12694,7 @@
         <v>10</v>
       </c>
       <c r="F413" s="1">
-        <v>999.93695417449999</v>
+        <v>200</v>
       </c>
       <c r="G413" t="s">
         <v>503</v>
@@ -12763,7 +12763,7 @@
         <v>10</v>
       </c>
       <c r="F416" s="1">
-        <v>796.08404240000004</v>
+        <v>200</v>
       </c>
       <c r="G416" t="s">
         <v>713</v>
@@ -12809,7 +12809,7 @@
         <v>10</v>
       </c>
       <c r="F418" s="1">
-        <v>477.73829419999998</v>
+        <v>200</v>
       </c>
       <c r="G418" t="s">
         <v>614</v>
@@ -12878,7 +12878,7 @@
         <v>10</v>
       </c>
       <c r="F421" s="1">
-        <v>965.99270811999997</v>
+        <v>200</v>
       </c>
       <c r="G421" t="s">
         <v>388</v>
@@ -12947,7 +12947,7 @@
         <v>10</v>
       </c>
       <c r="F424" s="1">
-        <v>625.78333000000009</v>
+        <v>200</v>
       </c>
       <c r="G424" t="s">
         <v>936</v>
@@ -12993,7 +12993,7 @@
         <v>10</v>
       </c>
       <c r="F426" s="1">
-        <v>1749.8111215200001</v>
+        <v>200</v>
       </c>
       <c r="G426" t="s">
         <v>936</v>
@@ -13016,7 +13016,7 @@
         <v>10</v>
       </c>
       <c r="F427" s="1">
-        <v>902.11881140000003</v>
+        <v>200</v>
       </c>
       <c r="G427" t="s">
         <v>936</v>
@@ -13039,7 +13039,7 @@
         <v>10</v>
       </c>
       <c r="F428" s="1">
-        <v>670.18511749999993</v>
+        <v>200</v>
       </c>
       <c r="G428" t="s">
         <v>936</v>
@@ -13062,7 +13062,7 @@
         <v>10</v>
       </c>
       <c r="F429" s="1">
-        <v>664.36645659999988</v>
+        <v>200</v>
       </c>
       <c r="G429" t="s">
         <v>936</v>
@@ -13131,7 +13131,7 @@
         <v>10</v>
       </c>
       <c r="F432" s="1">
-        <v>612.83374890000005</v>
+        <v>200</v>
       </c>
       <c r="G432" t="s">
         <v>936</v>
@@ -13200,7 +13200,7 @@
         <v>10</v>
       </c>
       <c r="F435" s="1">
-        <v>698.67212070000005</v>
+        <v>200</v>
       </c>
       <c r="G435" t="s">
         <v>936</v>
@@ -13246,7 +13246,7 @@
         <v>10</v>
       </c>
       <c r="F437" s="1">
-        <v>610.90643929999999</v>
+        <v>200</v>
       </c>
       <c r="G437" t="s">
         <v>936</v>
@@ -13315,7 +13315,7 @@
         <v>10</v>
       </c>
       <c r="F440" s="1">
-        <v>901.22275335999996</v>
+        <v>200</v>
       </c>
       <c r="G440" t="s">
         <v>936</v>
@@ -13384,7 +13384,7 @@
         <v>10</v>
       </c>
       <c r="F443" s="1">
-        <v>1742.70296426</v>
+        <v>200</v>
       </c>
       <c r="G443" t="s">
         <v>651</v>
@@ -13499,7 +13499,7 @@
         <v>10</v>
       </c>
       <c r="F448" s="1">
-        <v>620.73520069999995</v>
+        <v>200</v>
       </c>
       <c r="G448" t="s">
         <v>713</v>
@@ -13660,7 +13660,7 @@
         <v>10</v>
       </c>
       <c r="F455" s="1">
-        <v>1740.04578414</v>
+        <v>200</v>
       </c>
       <c r="G455" t="s">
         <v>644</v>
@@ -13706,7 +13706,7 @@
         <v>10</v>
       </c>
       <c r="F457" s="1">
-        <v>676.97858419999989</v>
+        <v>200</v>
       </c>
       <c r="G457" t="s">
         <v>644</v>
@@ -13775,7 +13775,7 @@
         <v>10</v>
       </c>
       <c r="F460" s="1">
-        <v>887.57326</v>
+        <v>200</v>
       </c>
       <c r="G460" t="s">
         <v>687</v>
@@ -13821,7 +13821,7 @@
         <v>10</v>
       </c>
       <c r="F462" s="1">
-        <v>984.66313272999992</v>
+        <v>200</v>
       </c>
       <c r="G462" t="s">
         <v>388</v>
@@ -13890,7 +13890,7 @@
         <v>10</v>
       </c>
       <c r="F465" s="1">
-        <v>1490.2113087</v>
+        <v>200</v>
       </c>
       <c r="G465" t="s">
         <v>651</v>
@@ -13959,7 +13959,7 @@
         <v>10</v>
       </c>
       <c r="F468" s="1">
-        <v>409.77413030000002</v>
+        <v>200</v>
       </c>
       <c r="G468" t="s">
         <v>651</v>
@@ -14074,7 +14074,7 @@
         <v>10</v>
       </c>
       <c r="F473" s="1">
-        <v>498.33411219999999</v>
+        <v>200</v>
       </c>
       <c r="G473" t="s">
         <v>651</v>
@@ -14143,7 +14143,7 @@
         <v>10</v>
       </c>
       <c r="F476" s="1">
-        <v>924.24464470000009</v>
+        <v>200</v>
       </c>
       <c r="G476" t="s">
         <v>651</v>
@@ -14189,7 +14189,7 @@
         <v>10</v>
       </c>
       <c r="F478" s="1">
-        <v>795.60904973970003</v>
+        <v>200</v>
       </c>
       <c r="G478" t="s">
         <v>651</v>
@@ -14281,7 +14281,7 @@
         <v>10</v>
       </c>
       <c r="F482" s="1">
-        <v>220.80562851000002</v>
+        <v>200</v>
       </c>
       <c r="G482" t="s">
         <v>408</v>
@@ -14304,7 +14304,7 @@
         <v>10</v>
       </c>
       <c r="F483" s="1">
-        <v>745.82143929999995</v>
+        <v>200</v>
       </c>
       <c r="G483" t="s">
         <v>651</v>
@@ -14373,7 +14373,7 @@
         <v>10</v>
       </c>
       <c r="F486" s="1">
-        <v>902.77834251000002</v>
+        <v>200</v>
       </c>
       <c r="G486" t="s">
         <v>351</v>
@@ -14511,7 +14511,7 @@
         <v>10</v>
       </c>
       <c r="F492" s="1">
-        <v>883.62291549999998</v>
+        <v>200</v>
       </c>
       <c r="G492" t="s">
         <v>408</v>
@@ -14557,7 +14557,7 @@
         <v>10</v>
       </c>
       <c r="F494" s="1">
-        <v>836.0904706</v>
+        <v>200</v>
       </c>
       <c r="G494" t="s">
         <v>651</v>
@@ -14764,7 +14764,7 @@
         <v>10</v>
       </c>
       <c r="F503" s="1">
-        <v>936.62447158999998</v>
+        <v>200</v>
       </c>
       <c r="G503" t="s">
         <v>429</v>
@@ -14856,7 +14856,7 @@
         <v>10</v>
       </c>
       <c r="F507" s="1">
-        <v>785.68593450000003</v>
+        <v>200</v>
       </c>
       <c r="G507" t="s">
         <v>713</v>
@@ -15063,7 +15063,7 @@
         <v>10</v>
       </c>
       <c r="F516" s="1">
-        <v>835.59179010000003</v>
+        <v>200</v>
       </c>
       <c r="G516" t="s">
         <v>687</v>
@@ -15109,7 +15109,7 @@
         <v>10</v>
       </c>
       <c r="F518" s="1">
-        <v>940.90238889000011</v>
+        <v>200</v>
       </c>
       <c r="G518" t="s">
         <v>687</v>
@@ -15155,7 +15155,7 @@
         <v>10</v>
       </c>
       <c r="F520" s="1">
-        <v>916.01444383</v>
+        <v>200</v>
       </c>
       <c r="G520" t="s">
         <v>687</v>
@@ -15201,7 +15201,7 @@
         <v>10</v>
       </c>
       <c r="F522" s="1">
-        <v>296.59854940000002</v>
+        <v>200</v>
       </c>
       <c r="G522" t="s">
         <v>687</v>
@@ -15293,7 +15293,7 @@
         <v>10</v>
       </c>
       <c r="F526" s="1">
-        <v>890.39028020000001</v>
+        <v>200</v>
       </c>
       <c r="G526" t="s">
         <v>687</v>
@@ -15339,7 +15339,7 @@
         <v>10</v>
       </c>
       <c r="F528" s="1">
-        <v>714.5261784999999</v>
+        <v>200</v>
       </c>
       <c r="G528" t="s">
         <v>687</v>
@@ -15385,7 +15385,7 @@
         <v>10</v>
       </c>
       <c r="F530" s="1">
-        <v>861.94637030000001</v>
+        <v>200</v>
       </c>
       <c r="G530" t="s">
         <v>687</v>
@@ -15408,7 +15408,7 @@
         <v>10</v>
       </c>
       <c r="F531" s="1">
-        <v>980.11560126999996</v>
+        <v>200</v>
       </c>
       <c r="G531" t="s">
         <v>687</v>
@@ -15454,7 +15454,7 @@
         <v>10</v>
       </c>
       <c r="F533" s="1">
-        <v>772.38746690000005</v>
+        <v>200</v>
       </c>
       <c r="G533" t="s">
         <v>687</v>
@@ -15500,7 +15500,7 @@
         <v>10</v>
       </c>
       <c r="F535" s="1">
-        <v>881.58829000000003</v>
+        <v>200</v>
       </c>
       <c r="G535" t="s">
         <v>687</v>
@@ -15523,7 +15523,7 @@
         <v>10</v>
       </c>
       <c r="F536" s="1">
-        <v>960.07980021000003</v>
+        <v>200</v>
       </c>
       <c r="G536" t="s">
         <v>687</v>
@@ -15546,7 +15546,7 @@
         <v>10</v>
       </c>
       <c r="F537" s="1">
-        <v>891.28652049999994</v>
+        <v>200</v>
       </c>
       <c r="G537" t="s">
         <v>687</v>
@@ -15592,7 +15592,7 @@
         <v>10</v>
       </c>
       <c r="F539" s="1">
-        <v>913.92358591999994</v>
+        <v>200</v>
       </c>
       <c r="G539" t="s">
         <v>687</v>
@@ -15638,7 +15638,7 @@
         <v>10</v>
       </c>
       <c r="F541" s="1">
-        <v>890.32251810000002</v>
+        <v>200</v>
       </c>
       <c r="G541" t="s">
         <v>687</v>
@@ -15661,7 +15661,7 @@
         <v>10</v>
       </c>
       <c r="F542" s="1">
-        <v>812.64751249999995</v>
+        <v>200</v>
       </c>
       <c r="G542" t="s">
         <v>687</v>
@@ -15684,7 +15684,7 @@
         <v>10</v>
       </c>
       <c r="F543" s="1">
-        <v>943.58032947999993</v>
+        <v>200</v>
       </c>
       <c r="G543" t="s">
         <v>408</v>
@@ -15707,7 +15707,7 @@
         <v>10</v>
       </c>
       <c r="F544" s="1">
-        <v>669.13658729999997</v>
+        <v>200</v>
       </c>
       <c r="G544" t="s">
         <v>651</v>
@@ -15845,7 +15845,7 @@
         <v>10</v>
       </c>
       <c r="F550" s="1">
-        <v>804.39346409999996</v>
+        <v>200</v>
       </c>
       <c r="G550" t="s">
         <v>713</v>
@@ -15914,7 +15914,7 @@
         <v>10</v>
       </c>
       <c r="F553" s="1">
-        <v>276.50980140000001</v>
+        <v>200</v>
       </c>
       <c r="G553" t="s">
         <v>713</v>
@@ -16052,7 +16052,7 @@
         <v>10</v>
       </c>
       <c r="F559" s="1">
-        <v>778.25793920000001</v>
+        <v>200</v>
       </c>
       <c r="G559" t="s">
         <v>713</v>
@@ -16098,7 +16098,7 @@
         <v>10</v>
       </c>
       <c r="F561" s="1">
-        <v>597.81907269999999</v>
+        <v>200</v>
       </c>
       <c r="G561" t="s">
         <v>713</v>
@@ -16121,7 +16121,7 @@
         <v>10</v>
       </c>
       <c r="F562" s="1">
-        <v>850.47247430000004</v>
+        <v>200</v>
       </c>
       <c r="G562" t="s">
         <v>713</v>
@@ -16167,7 +16167,7 @@
         <v>10</v>
       </c>
       <c r="F564" s="1">
-        <v>848.5983549</v>
+        <v>200</v>
       </c>
       <c r="G564" t="s">
         <v>713</v>
@@ -16282,7 +16282,7 @@
         <v>10</v>
       </c>
       <c r="F569" s="1">
-        <v>963.40701191000005</v>
+        <v>200</v>
       </c>
       <c r="G569" t="s">
         <v>713</v>
@@ -16466,7 +16466,7 @@
         <v>10</v>
       </c>
       <c r="F577" s="1">
-        <v>752.09018470000001</v>
+        <v>200</v>
       </c>
       <c r="G577" t="s">
         <v>713</v>
@@ -16604,7 +16604,7 @@
         <v>10</v>
       </c>
       <c r="F583" s="1">
-        <v>1909.4116194799999</v>
+        <v>200</v>
       </c>
       <c r="G583" t="s">
         <v>713</v>
@@ -16650,7 +16650,7 @@
         <v>10</v>
       </c>
       <c r="F585" s="1">
-        <v>510.32187190000002</v>
+        <v>200</v>
       </c>
       <c r="G585" t="s">
         <v>713</v>
@@ -16696,7 +16696,7 @@
         <v>10</v>
       </c>
       <c r="F587" s="1">
-        <v>774.88239429999999</v>
+        <v>200</v>
       </c>
       <c r="G587" t="s">
         <v>713</v>
@@ -16788,7 +16788,7 @@
         <v>10</v>
       </c>
       <c r="F591" s="1">
-        <v>750.49245080000003</v>
+        <v>200</v>
       </c>
       <c r="G591" t="s">
         <v>713</v>
@@ -16811,7 +16811,7 @@
         <v>10</v>
       </c>
       <c r="F592" s="1">
-        <v>948.13293259</v>
+        <v>200</v>
       </c>
       <c r="G592" t="s">
         <v>713</v>
@@ -16880,7 +16880,7 @@
         <v>10</v>
       </c>
       <c r="F595" s="1">
-        <v>946.51922569999999</v>
+        <v>200</v>
       </c>
       <c r="G595" t="s">
         <v>713</v>
@@ -16903,7 +16903,7 @@
         <v>10</v>
       </c>
       <c r="F596" s="1">
-        <v>3316.7621290000002</v>
+        <v>200</v>
       </c>
       <c r="G596" t="s">
         <v>713</v>
@@ -16995,7 +16995,7 @@
         <v>10</v>
       </c>
       <c r="F600" s="1">
-        <v>891.1014222</v>
+        <v>200</v>
       </c>
       <c r="G600" t="s">
         <v>420</v>
@@ -17110,7 +17110,7 @@
         <v>10</v>
       </c>
       <c r="F605" s="1">
-        <v>521.51504220000004</v>
+        <v>200</v>
       </c>
       <c r="G605" t="s">
         <v>753</v>
@@ -17156,7 +17156,7 @@
         <v>10</v>
       </c>
       <c r="F607" s="1">
-        <v>888.91374350000001</v>
+        <v>200</v>
       </c>
       <c r="G607" t="s">
         <v>753</v>
@@ -17179,7 +17179,7 @@
         <v>10</v>
       </c>
       <c r="F608" s="1">
-        <v>855.08684349999999</v>
+        <v>200</v>
       </c>
       <c r="G608" t="s">
         <v>713</v>
@@ -17202,7 +17202,7 @@
         <v>10</v>
       </c>
       <c r="F609" s="1">
-        <v>806.35136690000002</v>
+        <v>200</v>
       </c>
       <c r="G609" t="s">
         <v>529</v>
@@ -17248,7 +17248,7 @@
         <v>10</v>
       </c>
       <c r="F611" s="1">
-        <v>907.84964728</v>
+        <v>200</v>
       </c>
       <c r="G611" t="s">
         <v>529</v>
@@ -17386,7 +17386,7 @@
         <v>10</v>
       </c>
       <c r="F617" s="1">
-        <v>923.63043255000002</v>
+        <v>200</v>
       </c>
       <c r="G617" t="s">
         <v>762</v>
@@ -17478,7 +17478,7 @@
         <v>10</v>
       </c>
       <c r="F621" s="1">
-        <v>794.20607489999998</v>
+        <v>200</v>
       </c>
       <c r="G621" t="s">
         <v>855</v>
@@ -17570,7 +17570,7 @@
         <v>10</v>
       </c>
       <c r="F625" s="1">
-        <v>599.03029460000005</v>
+        <v>200</v>
       </c>
       <c r="G625" t="s">
         <v>651</v>
@@ -17616,7 +17616,7 @@
         <v>10</v>
       </c>
       <c r="F627" s="1">
-        <v>975.08791464000001</v>
+        <v>200</v>
       </c>
       <c r="G627" t="s">
         <v>687</v>
@@ -17639,7 +17639,7 @@
         <v>10</v>
       </c>
       <c r="F628" s="1">
-        <v>901.21541080999998</v>
+        <v>200</v>
       </c>
       <c r="G628" t="s">
         <v>777</v>
@@ -17685,7 +17685,7 @@
         <v>10</v>
       </c>
       <c r="F630" s="1">
-        <v>878.37595729999998</v>
+        <v>200</v>
       </c>
       <c r="G630" t="s">
         <v>777</v>
@@ -17731,7 +17731,7 @@
         <v>10</v>
       </c>
       <c r="F632" s="1">
-        <v>825.27720610000006</v>
+        <v>200</v>
       </c>
       <c r="G632" t="s">
         <v>777</v>
@@ -17777,7 +17777,7 @@
         <v>10</v>
       </c>
       <c r="F634" s="1">
-        <v>474.06389399999995</v>
+        <v>200</v>
       </c>
       <c r="G634" t="s">
         <v>777</v>
@@ -17823,7 +17823,7 @@
         <v>10</v>
       </c>
       <c r="F636" s="1">
-        <v>670.3407365999999</v>
+        <v>200</v>
       </c>
       <c r="G636" t="s">
         <v>777</v>
@@ -17869,7 +17869,7 @@
         <v>10</v>
       </c>
       <c r="F638" s="1">
-        <v>292.77526556799995</v>
+        <v>200</v>
       </c>
       <c r="G638" t="s">
         <v>777</v>
@@ -17892,7 +17892,7 @@
         <v>10</v>
       </c>
       <c r="F639" s="1">
-        <v>570.66732239999999</v>
+        <v>200</v>
       </c>
       <c r="G639" t="s">
         <v>777</v>
@@ -17938,7 +17938,7 @@
         <v>10</v>
       </c>
       <c r="F641" s="1">
-        <v>807.32017680000001</v>
+        <v>200</v>
       </c>
       <c r="G641" t="s">
         <v>777</v>
@@ -18007,7 +18007,7 @@
         <v>10</v>
       </c>
       <c r="F644" s="1">
-        <v>886.09659039999997</v>
+        <v>200</v>
       </c>
       <c r="G644" t="s">
         <v>777</v>
@@ -18076,7 +18076,7 @@
         <v>10</v>
       </c>
       <c r="F647" s="1">
-        <v>1583.7098785000001</v>
+        <v>200</v>
       </c>
       <c r="G647" t="s">
         <v>918</v>
@@ -18145,7 +18145,7 @@
         <v>10</v>
       </c>
       <c r="F650" s="1">
-        <v>703.95900259999996</v>
+        <v>200</v>
       </c>
       <c r="G650" t="s">
         <v>713</v>
@@ -18260,7 +18260,7 @@
         <v>10</v>
       </c>
       <c r="F655" s="1">
-        <v>812.43273470000008</v>
+        <v>200</v>
       </c>
       <c r="G655" t="s">
         <v>788</v>
@@ -18329,7 +18329,7 @@
         <v>10</v>
       </c>
       <c r="F658" s="1">
-        <v>575.48161085000004</v>
+        <v>200</v>
       </c>
       <c r="G658" t="s">
         <v>788</v>
@@ -18444,7 +18444,7 @@
         <v>10</v>
       </c>
       <c r="F663" s="1">
-        <v>238.74579070000001</v>
+        <v>200</v>
       </c>
       <c r="G663" t="s">
         <v>429</v>
@@ -18467,7 +18467,7 @@
         <v>10</v>
       </c>
       <c r="F664" s="1">
-        <v>361.85275120000011</v>
+        <v>200</v>
       </c>
       <c r="G664" t="s">
         <v>651</v>
@@ -18513,7 +18513,7 @@
         <v>10</v>
       </c>
       <c r="F666" s="1">
-        <v>745.91120269999999</v>
+        <v>200</v>
       </c>
       <c r="G666" t="s">
         <v>800</v>
@@ -18582,7 +18582,7 @@
         <v>10</v>
       </c>
       <c r="F669" s="1">
-        <v>805.73714910000001</v>
+        <v>200</v>
       </c>
       <c r="G669" t="s">
         <v>800</v>
@@ -18628,7 +18628,7 @@
         <v>10</v>
       </c>
       <c r="F671" s="1">
-        <v>614.60316910000006</v>
+        <v>200</v>
       </c>
       <c r="G671" t="s">
         <v>800</v>
@@ -18674,7 +18674,7 @@
         <v>10</v>
       </c>
       <c r="F673" s="1">
-        <v>581.21419689999993</v>
+        <v>200</v>
       </c>
       <c r="G673" t="s">
         <v>800</v>
@@ -18720,7 +18720,7 @@
         <v>10</v>
       </c>
       <c r="F675" s="1">
-        <v>839.14304850000008</v>
+        <v>200</v>
       </c>
       <c r="G675" t="s">
         <v>651</v>
@@ -18766,7 +18766,7 @@
         <v>10</v>
       </c>
       <c r="F677" s="1">
-        <v>970.21007995000002</v>
+        <v>200</v>
       </c>
       <c r="G677" t="s">
         <v>918</v>
@@ -18812,7 +18812,7 @@
         <v>10</v>
       </c>
       <c r="F679" s="1">
-        <v>765.28043749999995</v>
+        <v>200</v>
       </c>
       <c r="G679" t="s">
         <v>803</v>
@@ -18858,7 +18858,7 @@
         <v>10</v>
       </c>
       <c r="F681" s="1">
-        <v>875.70736390000002</v>
+        <v>200</v>
       </c>
       <c r="G681" t="s">
         <v>420</v>
@@ -18904,7 +18904,7 @@
         <v>10</v>
       </c>
       <c r="F683" s="1">
-        <v>906.94340807999993</v>
+        <v>200</v>
       </c>
       <c r="G683" t="s">
         <v>806</v>
@@ -18973,7 +18973,7 @@
         <v>10</v>
       </c>
       <c r="F686" s="1">
-        <v>798.79990880000003</v>
+        <v>200</v>
       </c>
       <c r="G686" t="s">
         <v>519</v>
@@ -19042,7 +19042,7 @@
         <v>10</v>
       </c>
       <c r="F689" s="1">
-        <v>1549.9198371100001</v>
+        <v>200</v>
       </c>
       <c r="G689" t="s">
         <v>848</v>
@@ -19088,7 +19088,7 @@
         <v>10</v>
       </c>
       <c r="F691" s="1">
-        <v>908.94535736</v>
+        <v>200</v>
       </c>
       <c r="G691" t="s">
         <v>855</v>
@@ -19157,7 +19157,7 @@
         <v>10</v>
       </c>
       <c r="F694" s="1">
-        <v>841.22559909999995</v>
+        <v>200</v>
       </c>
       <c r="G694" t="s">
         <v>855</v>
@@ -19226,7 +19226,7 @@
         <v>10</v>
       </c>
       <c r="F697" s="1">
-        <v>1773.2559402109998</v>
+        <v>200</v>
       </c>
       <c r="G697" t="s">
         <v>848</v>
@@ -19295,7 +19295,7 @@
         <v>10</v>
       </c>
       <c r="F700" s="1">
-        <v>1619.3486707000002</v>
+        <v>200</v>
       </c>
       <c r="G700" t="s">
         <v>848</v>
@@ -19364,7 +19364,7 @@
         <v>10</v>
       </c>
       <c r="F703" s="1">
-        <v>950.14880102999996</v>
+        <v>200</v>
       </c>
       <c r="G703" t="s">
         <v>841</v>
@@ -19433,7 +19433,7 @@
         <v>10</v>
       </c>
       <c r="F706" s="1">
-        <v>907.80785026000001</v>
+        <v>200</v>
       </c>
       <c r="G706" t="s">
         <v>855</v>
@@ -19525,7 +19525,7 @@
         <v>10</v>
       </c>
       <c r="F710" s="1">
-        <v>288.83042890000013</v>
+        <v>200</v>
       </c>
       <c r="G710" t="s">
         <v>855</v>
@@ -19640,7 +19640,7 @@
         <v>10</v>
       </c>
       <c r="F715" s="1">
-        <v>1538.3066934199999</v>
+        <v>200</v>
       </c>
       <c r="G715" t="s">
         <v>848</v>
@@ -19755,7 +19755,7 @@
         <v>10</v>
       </c>
       <c r="F720" s="1">
-        <v>1398.3826650200001</v>
+        <v>200</v>
       </c>
       <c r="G720" t="s">
         <v>855</v>
@@ -19847,7 +19847,7 @@
         <v>10</v>
       </c>
       <c r="F724" s="1">
-        <v>958.32861328000001</v>
+        <v>200</v>
       </c>
       <c r="G724" t="s">
         <v>848</v>
@@ -19893,7 +19893,7 @@
         <v>10</v>
       </c>
       <c r="F726" s="1">
-        <v>461.80297769999999</v>
+        <v>200</v>
       </c>
       <c r="G726" t="s">
         <v>841</v>
@@ -19985,7 +19985,7 @@
         <v>10</v>
       </c>
       <c r="F730" s="1">
-        <v>1999.349285937187</v>
+        <v>200</v>
       </c>
       <c r="G730" t="s">
         <v>855</v>
@@ -20054,7 +20054,7 @@
         <v>10</v>
       </c>
       <c r="F733" s="1">
-        <v>1666.8227980060001</v>
+        <v>200</v>
       </c>
       <c r="G733" t="s">
         <v>846</v>
@@ -20123,7 +20123,7 @@
         <v>10</v>
       </c>
       <c r="F736" s="1">
-        <v>384.88526040000005</v>
+        <v>200</v>
       </c>
       <c r="G736" t="s">
         <v>848</v>
@@ -20169,7 +20169,7 @@
         <v>10</v>
       </c>
       <c r="F738" s="1">
-        <v>762.27662789999999</v>
+        <v>200</v>
       </c>
       <c r="G738" t="s">
         <v>848</v>
@@ -20238,7 +20238,7 @@
         <v>10</v>
       </c>
       <c r="F741" s="1">
-        <v>775.482845</v>
+        <v>200</v>
       </c>
       <c r="G741" t="s">
         <v>848</v>
@@ -20330,7 +20330,7 @@
         <v>10</v>
       </c>
       <c r="F745" s="1">
-        <v>993.77827885300007</v>
+        <v>200</v>
       </c>
       <c r="G745" t="s">
         <v>855</v>
@@ -20376,7 +20376,7 @@
         <v>10</v>
       </c>
       <c r="F747" s="1">
-        <v>755.98855609999998</v>
+        <v>200</v>
       </c>
       <c r="G747" t="s">
         <v>846</v>
@@ -20629,7 +20629,7 @@
         <v>10</v>
       </c>
       <c r="F758" s="1">
-        <v>1720.2355098100002</v>
+        <v>200</v>
       </c>
       <c r="G758" t="s">
         <v>848</v>
@@ -20813,7 +20813,7 @@
         <v>10</v>
       </c>
       <c r="F766" s="1">
-        <v>459.58643259999991</v>
+        <v>200</v>
       </c>
       <c r="G766" t="s">
         <v>873</v>
@@ -20882,7 +20882,7 @@
         <v>10</v>
       </c>
       <c r="F769" s="1">
-        <v>894.02989280000008</v>
+        <v>200</v>
       </c>
       <c r="G769" t="s">
         <v>420</v>
@@ -20974,7 +20974,7 @@
         <v>10</v>
       </c>
       <c r="F773" s="1">
-        <v>322.12289829999997</v>
+        <v>200</v>
       </c>
       <c r="G773" t="s">
         <v>878</v>
@@ -21043,7 +21043,7 @@
         <v>10</v>
       </c>
       <c r="F776" s="1">
-        <v>794.70891370000004</v>
+        <v>200</v>
       </c>
       <c r="G776" t="s">
         <v>841</v>
@@ -21066,7 +21066,7 @@
         <v>10</v>
       </c>
       <c r="F777" s="1">
-        <v>709.8271029</v>
+        <v>200</v>
       </c>
       <c r="G777" t="s">
         <v>855</v>
@@ -21089,7 +21089,7 @@
         <v>10</v>
       </c>
       <c r="F778" s="1">
-        <v>402.79238050000004</v>
+        <v>200</v>
       </c>
       <c r="G778" t="s">
         <v>395</v>
@@ -21227,7 +21227,7 @@
         <v>10</v>
       </c>
       <c r="F784" s="1">
-        <v>879.87076549999995</v>
+        <v>200</v>
       </c>
       <c r="G784" t="s">
         <v>519</v>
@@ -21296,7 +21296,7 @@
         <v>10</v>
       </c>
       <c r="F787" s="1">
-        <v>920.37786187000006</v>
+        <v>200</v>
       </c>
       <c r="G787" t="s">
         <v>937</v>
@@ -21342,7 +21342,7 @@
         <v>10</v>
       </c>
       <c r="F789" s="1">
-        <v>950.80491830000005</v>
+        <v>200</v>
       </c>
       <c r="G789" t="s">
         <v>937</v>
@@ -21365,7 +21365,7 @@
         <v>10</v>
       </c>
       <c r="F790" s="1">
-        <v>804.16690459999995</v>
+        <v>200</v>
       </c>
       <c r="G790" t="s">
         <v>937</v>
@@ -21411,7 +21411,7 @@
         <v>10</v>
       </c>
       <c r="F792" s="1">
-        <v>908.40698140999996</v>
+        <v>200</v>
       </c>
       <c r="G792" t="s">
         <v>937</v>
@@ -21457,7 +21457,7 @@
         <v>10</v>
       </c>
       <c r="F794" s="1">
-        <v>891.95152329999996</v>
+        <v>200</v>
       </c>
       <c r="G794" t="s">
         <v>937</v>
@@ -21526,7 +21526,7 @@
         <v>10</v>
       </c>
       <c r="F797" s="1">
-        <v>940.85806272000002</v>
+        <v>200</v>
       </c>
       <c r="G797" t="s">
         <v>937</v>
@@ -21572,7 +21572,7 @@
         <v>10</v>
       </c>
       <c r="F799" s="1">
-        <v>897.23087610000005</v>
+        <v>200</v>
       </c>
       <c r="G799" t="s">
         <v>937</v>
@@ -21595,7 +21595,7 @@
         <v>10</v>
       </c>
       <c r="F800" s="1">
-        <v>709.33554019999997</v>
+        <v>200</v>
       </c>
       <c r="G800" t="s">
         <v>788</v>
@@ -21641,7 +21641,7 @@
         <v>10</v>
       </c>
       <c r="F802" s="1">
-        <v>577.97541130000002</v>
+        <v>200</v>
       </c>
       <c r="G802" t="s">
         <v>899</v>
@@ -21687,7 +21687,7 @@
         <v>10</v>
       </c>
       <c r="F804" s="1">
-        <v>466.94834939999987</v>
+        <v>200</v>
       </c>
       <c r="G804" t="s">
         <v>899</v>
@@ -21710,7 +21710,7 @@
         <v>10</v>
       </c>
       <c r="F805" s="1">
-        <v>410.2959323</v>
+        <v>200</v>
       </c>
       <c r="G805" t="s">
         <v>899</v>
@@ -21802,7 +21802,7 @@
         <v>10</v>
       </c>
       <c r="F809" s="1">
-        <v>694.36902569999995</v>
+        <v>200</v>
       </c>
       <c r="G809" t="s">
         <v>899</v>
@@ -21871,7 +21871,7 @@
         <v>10</v>
       </c>
       <c r="F812" s="1">
-        <v>720.62479180000003</v>
+        <v>200</v>
       </c>
       <c r="G812" t="s">
         <v>420</v>
@@ -21917,7 +21917,7 @@
         <v>10</v>
       </c>
       <c r="F814" s="1">
-        <v>229.3992537</v>
+        <v>200</v>
       </c>
       <c r="G814" t="s">
         <v>777</v>
@@ -21940,7 +21940,7 @@
         <v>10</v>
       </c>
       <c r="F815" s="1">
-        <v>704.19455169999992</v>
+        <v>200</v>
       </c>
       <c r="G815" t="s">
         <v>351</v>
@@ -22032,7 +22032,7 @@
         <v>10</v>
       </c>
       <c r="F819" s="1">
-        <v>984.02699276999999</v>
+        <v>200</v>
       </c>
       <c r="G819" t="s">
         <v>388</v>
@@ -22170,7 +22170,7 @@
         <v>10</v>
       </c>
       <c r="F825" s="1">
-        <v>818.31216830000005</v>
+        <v>200</v>
       </c>
       <c r="G825" t="s">
         <v>918</v>
@@ -22262,7 +22262,7 @@
         <v>10</v>
       </c>
       <c r="F829" s="1">
-        <v>991.98757905599996</v>
+        <v>200</v>
       </c>
       <c r="G829" t="s">
         <v>918</v>
@@ -22308,7 +22308,7 @@
         <v>10</v>
       </c>
       <c r="F831" s="1">
-        <v>1778.9839817</v>
+        <v>200</v>
       </c>
       <c r="G831" t="s">
         <v>918</v>
@@ -22331,7 +22331,7 @@
         <v>10</v>
       </c>
       <c r="F832" s="1">
-        <v>868.42514510000001</v>
+        <v>200</v>
       </c>
       <c r="G832" t="s">
         <v>918</v>
@@ -22377,7 +22377,7 @@
         <v>10</v>
       </c>
       <c r="F834" s="1">
-        <v>879.62511600000005</v>
+        <v>200</v>
       </c>
       <c r="G834" t="s">
         <v>918</v>

</xml_diff>